<commit_message>
chore: run 2026-05-07 09:26 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_07_05_2026.xlsx
+++ b/logs/Consolidado_07_05_2026.xlsx
@@ -641,7 +641,7 @@
         <v>14</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -660,7 +660,7 @@
         <v>29</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -695,10 +695,10 @@
         <v>68</v>
       </c>
       <c r="C5" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -714,10 +714,10 @@
         <v>46</v>
       </c>
       <c r="C6" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>3</v>
@@ -733,10 +733,10 @@
         <v>97</v>
       </c>
       <c r="C7" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>15</v>
@@ -752,10 +752,10 @@
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -856,7 +856,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>6179447</t>
+        </is>
+      </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>25%</t>
@@ -15091,40 +15095,40 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>Okara Blond Brightening Shampoo Blond Hair
 Champô Iluminador Louro Natural ou Pintado
 200 ml</t>
         </is>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/okara-blond-brightening-shampoo-blond-hair-6760061.html</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr"/>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr"/>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>6760061</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -15171,40 +15175,40 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>Okara Silver Toning Shampoo
 Champô Violeta Cabelo Branco Grisalho ou Louro
 200 ml</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/okara-silver-toning-shampoo-6759950.html</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr"/>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>6759950</t>
         </is>
       </c>
-      <c r="H36" s="7" t="inlineStr">
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -16846,40 +16850,40 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Biology AC Perfect Anti-Blemish Fluid
 Creme Fluído Marcas Acne Ácido Hialurónico
 40 ml</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/biology-ac-perfect-anti-blemish-fluid-7756130.html</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>7756130</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -17295,43 +17299,43 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Dermalibour+ Repairing CICA-Cream
 Creme Reparador Purificante Pele Irritada</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/dermalibour-repairing-cica-cream-452821.html</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>7434602</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -18764,40 +18768,40 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>Protect AC Mattifying Fluid SPF50+
 Protetor Solar Fluido Mate Rosto Pele Oleosa
 40ml</t>
         </is>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-ac-mattifying-fluid-spf50-5782463.html</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr"/>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="E50" s="3" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
         <is>
           <t>5782463</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H50" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -19043,40 +19047,40 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Protect Pocket Invisible Fluid SPF50+
 Protetor Solar Fluido Rosto Pele Oleosa
 30 ml</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-pocket-invisible-fluid-spf50-7755407.html</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr"/>
-      <c r="F57" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G57" s="7" t="inlineStr">
+      <c r="E57" s="5" t="inlineStr"/>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
         <is>
           <t>7755407</t>
         </is>
       </c>
-      <c r="H57" s="7" t="inlineStr">
+      <c r="H57" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -19123,40 +19127,40 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B59" s="7" t="inlineStr">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C59" s="7" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>Protect X-TREM Stick Invisible SPF50+
 Protetor Solar Corpo Rosto Lábios
 8 gr</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-x-trem-stick-invisible-spf50-7129109.html</t>
         </is>
       </c>
-      <c r="E59" s="7" t="inlineStr"/>
-      <c r="F59" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G59" s="7" t="inlineStr">
+      <c r="E59" s="5" t="inlineStr"/>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
         <is>
           <t>7129109</t>
         </is>
       </c>
-      <c r="H59" s="7" t="inlineStr">
+      <c r="H59" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -19353,17 +19357,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Eludril
 Care Colutório Antiplaca
@@ -19371,23 +19375,23 @@
 500 ml</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/care-colutorio-antiplaca-4963445.html</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>4963445</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Sem desconto</t>
         </is>
@@ -19716,40 +19720,40 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Elgydium
 Dentrifíco Sensileave Dentes Sensíveis
 50 ml</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/dentrifico-sensileave-dentes-sensiveis-7181157.html</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>7181157</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -19796,40 +19800,40 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Elgydium
 Elgydium Fix Fixação Forte
 45 g</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/elgydium-fix-fixacao-forte-7434256.html</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr"/>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>7434256</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -21362,40 +21366,40 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C53" s="7" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>Elgydium
 Escovilhões Clinic Mono Pretos
 4 un</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D53" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/escovilhoes-clinic-mono-pretos-6937302.html</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr"/>
-      <c r="F53" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr">
+      <c r="E53" s="5" t="inlineStr"/>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
         <is>
           <t>6937302</t>
         </is>
       </c>
-      <c r="H53" s="7" t="inlineStr">
+      <c r="H53" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -21963,40 +21967,40 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B68" s="7" t="inlineStr">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C68" s="7" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>Elgydium
 Gel Dentífrico Menta Suave 7-12 Anos
 50 ml</t>
         </is>
       </c>
-      <c r="D68" s="7" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/gel-dentifrico-menta-suave-7-12-anos-6865620.html</t>
         </is>
       </c>
-      <c r="E68" s="7" t="inlineStr"/>
-      <c r="F68" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G68" s="7" t="inlineStr">
+      <c r="E68" s="3" t="inlineStr"/>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
         <is>
           <t>6865620</t>
         </is>
       </c>
-      <c r="H68" s="7" t="inlineStr">
+      <c r="H68" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -22043,40 +22047,40 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B70" s="7" t="inlineStr">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C70" s="7" t="inlineStr">
+      <c r="C70" s="3" t="inlineStr">
         <is>
           <t>Elugel
 Gel Redutor Placa Bacteriana
 40 ml</t>
         </is>
       </c>
-      <c r="D70" s="7" t="inlineStr">
+      <c r="D70" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/gel-redutor-placa-bacteriana-3017892.html</t>
         </is>
       </c>
-      <c r="E70" s="7" t="inlineStr"/>
-      <c r="F70" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G70" s="7" t="inlineStr">
+      <c r="E70" s="3" t="inlineStr"/>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
         <is>
           <t>3017892</t>
         </is>
       </c>
-      <c r="H70" s="7" t="inlineStr">
+      <c r="H70" s="3" t="inlineStr">
         <is>
           <t>Sem desconto</t>
         </is>
@@ -22649,40 +22653,40 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B85" s="7" t="inlineStr">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C85" s="7" t="inlineStr">
+      <c r="C85" s="5" t="inlineStr">
         <is>
           <t>Elgydium
 Raspador de Língua Breath
 1 un</t>
         </is>
       </c>
-      <c r="D85" s="7" t="inlineStr">
+      <c r="D85" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/raspador-de-lingua-breath-8071465.html</t>
         </is>
       </c>
-      <c r="E85" s="7" t="inlineStr"/>
-      <c r="F85" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G85" s="7" t="inlineStr">
+      <c r="E85" s="5" t="inlineStr"/>
+      <c r="F85" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
         <is>
           <t>8071465</t>
         </is>
       </c>
-      <c r="H85" s="7" t="inlineStr">
+      <c r="H85" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -23493,40 +23497,40 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Dexeryl</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Creme Emoliente Pele Seca ou Atópica
 Creme Corpo para Pele Seca e Atópica
 250 gr</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/creme-emoliente-pele-seca-ou-atopica-6037808.html</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>6037808</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -23798,38 +23802,38 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Dermalibour+ Repairing CICA-Cream
 Creme Reparador Purificante Pele Irritada</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>7434602</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/dermalibour-repairing-cica-cream-452821.html</t>
         </is>

</xml_diff>

<commit_message>
chore: run 2026-05-07 14:08 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_07_05_2026.xlsx
+++ b/logs/Consolidado_07_05_2026.xlsx
@@ -638,7 +638,7 @@
         <v>147</v>
       </c>
       <c r="C2" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -657,7 +657,7 @@
         <v>66</v>
       </c>
       <c r="C3" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -676,7 +676,7 @@
         <v>70</v>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -695,7 +695,7 @@
         <v>68</v>
       </c>
       <c r="C5" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -714,7 +714,7 @@
         <v>46</v>
       </c>
       <c r="C6" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -733,10 +733,10 @@
         <v>97</v>
       </c>
       <c r="C7" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
         <v>15</v>
@@ -1148,39 +1148,39 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Body Gentle Shower Gel for Sensitive Skin
 Gel Duche Hidrata Rosto e Corpo Pele Sensível</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/body-gentle-shower-gel-for-sensitive-skin-443318.html</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>6545079</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -1918,40 +1918,40 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Cleanance Comedomed Peeling Cleansing Gel
 Gel de Limpeza esfoliante pele com Acne
 400 ml</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/cleanance-comedomed-peeling-cleansing-gel-8660052.html</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr"/>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>8660052</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -2563,40 +2563,40 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>Couvrance Fluid Foundation Corrector 3.0
 Base Fluída Corretora SPF20
 30ml</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/couvrance-fluid-foundation-corrector-3.0-3599509.html</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr"/>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="E45" s="5" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>3599509</t>
         </is>
       </c>
-      <c r="H45" s="7" t="inlineStr">
+      <c r="H45" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -3643,40 +3643,40 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B72" s="7" t="inlineStr">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C72" s="7" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
         <is>
           <t>Hydrance BB Light Tinted Hydrating Emulsion
 BB Cream Leve e Fluído Hidratante 24h SPF30
 40 ml</t>
         </is>
       </c>
-      <c r="D72" s="7" t="inlineStr">
+      <c r="D72" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/hydrance-bb-light-tinted-hydrating-emulsion-5731161.html</t>
         </is>
       </c>
-      <c r="E72" s="7" t="inlineStr"/>
-      <c r="F72" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G72" s="7" t="inlineStr">
+      <c r="E72" s="3" t="inlineStr"/>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
         <is>
           <t>5731161</t>
         </is>
       </c>
-      <c r="H72" s="7" t="inlineStr">
+      <c r="H72" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -6342,40 +6342,40 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B139" s="7" t="inlineStr">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C139" s="7" t="inlineStr">
+      <c r="C139" s="5" t="inlineStr">
         <is>
           <t>Ultra Serum Instantly Plumps SPF50+
 Protetor Solar Sérum Rosto AH+Niacinamida
 30 ml</t>
         </is>
       </c>
-      <c r="D139" s="7" t="inlineStr">
+      <c r="D139" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/ultra-serum-instantly-plumps-spf50-8784379.html</t>
         </is>
       </c>
-      <c r="E139" s="7" t="inlineStr"/>
-      <c r="F139" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G139" s="7" t="inlineStr">
+      <c r="E139" s="5" t="inlineStr"/>
+      <c r="F139" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G139" s="5" t="inlineStr">
         <is>
           <t>8784379</t>
         </is>
       </c>
-      <c r="H139" s="7" t="inlineStr">
+      <c r="H139" s="5" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
@@ -7389,40 +7389,40 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Anaphase Anti-Hair Loss Anti-Thinning
 Champô Queda de Cabelo Crónica
 400 ml</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/anaphase-anti-hair-loss-anti-thinning-5622007.html</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>5622007</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -7829,40 +7829,40 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Creme Tratamento do Eczema Dexyane
 Creme Reparador Trata Lesões de Eczema
 100 ml</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/creme-tratamento-do-eczema-dexyane-5976178.html</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr"/>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>5976178</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -9695,40 +9695,40 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C63" s="7" t="inlineStr">
+      <c r="C63" s="3" t="inlineStr">
         <is>
           <t>Refill Kelual Squanorm Moisturizing Treatment Shampoo
 Champô Hidratante Caspa Seca Recarga
 400 ml</t>
         </is>
       </c>
-      <c r="D63" s="7" t="inlineStr">
+      <c r="D63" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/refill-kelual-squanorm-moisturizing-treatment-shampoo-8710843.html</t>
         </is>
       </c>
-      <c r="E63" s="7" t="inlineStr"/>
-      <c r="F63" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G63" s="7" t="inlineStr">
+      <c r="E63" s="3" t="inlineStr"/>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
         <is>
           <t>8710843</t>
         </is>
       </c>
-      <c r="H63" s="7" t="inlineStr">
+      <c r="H63" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -10210,40 +10210,40 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Bebé Cleansing Lotion No-Rise
 Leite Limpeza Fralda e Mãos 0 meses
 500 ml</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/bebe-cleansing-lotion-no-rise-6661598.html</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr"/>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>6661598</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -10856,40 +10856,40 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Crème Solaire Sublime SPF 30
 Protetor Solar de Rosto Antienvelhecimento
 50 ml</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/creme-solaire-sublime-spf-30-7129218.html</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr"/>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>7129218</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -11255,43 +11255,43 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Flax Volume Fine Hair Shampoo
 Champô Fibras de Linho BIO Volume Cabelo Fino</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/flax-volume-fine-hair-shampoo-343984.html</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>5221797</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -11751,40 +11751,40 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>Huile Réparatrice Après-Soleil
 Óleo Protetor de Cabelo Nutritivo
 150 ml</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/huile-reparatrice-apres-soleil-7546027.html</t>
         </is>
       </c>
-      <c r="E40" s="7" t="inlineStr"/>
-      <c r="F40" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G40" s="7" t="inlineStr">
+      <c r="E40" s="3" t="inlineStr"/>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
         <is>
           <t>7546027</t>
         </is>
       </c>
-      <c r="H40" s="7" t="inlineStr">
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -13881,120 +13881,120 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>5 Sens Enhancing Shampoo Frequent Use
 Champô Sublimador Realça o Brilho
 250 ml</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/5-sens-enhancing-shampoo-frequent-use-6218353.html</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>6218353</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Absolue Kératine Renewal Care Serum
 Sérum Reparador Extremo Pontas Danificadas
 30 ml</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/absolue-keratine-renewal-care-serum-7447296.html</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>7447296</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>36%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Absolue Kératine Repairing Beauty Cream
 Creme Leave-In Reparador Cabelo Danificado
 100 ml</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/absolue-keratine-repairing-beauty-cream-6997974.html</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>6997974</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -14161,40 +14161,40 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Astera Fresh Soothing Freshness Shampoo
 Champô Calmante Couro Cabeludo Irritado
 200 ml</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/astera-fresh-soothing-freshness-shampoo-5520033.html</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>5520033</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -14281,40 +14281,40 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Color Glow Repairing Glow Conditioner
 Máscara Reparadora Cabelo Pintado e Madeixas
 200 ml</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/color-glow-repairing-glow-conditioner-7924433.html</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr"/>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>7924433</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -14401,40 +14401,40 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Forticea Energizing Lotion
 Loção Leave-In Fortificante Todos Tipo Cabelo
 100 ml</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/forticea-energizing-lotion-6490926.html</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr"/>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>6490926</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>28%</t>
         </is>
@@ -14607,80 +14607,80 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Head Spa Complexe 5 Essential Oils
 Pré-Champô Estimulante Revitalizante
 50 ml</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/head-spa-complexe-5-essential-oils-5558743.html</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr"/>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>5558743</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Head Spa Purifying Scrub Detox
 Esfoliante Pré-Champô Couro Cabeludo Oleoso
 150 ml</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/head-spa-purifying-scrub-detox-7824621.html</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr"/>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>7824621</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>33%</t>
         </is>
@@ -15015,40 +15015,40 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>Naturia Invisible Dry Shampoo
 Champô Seco Invisível Lavanda Orgânica
 75 ml</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/naturia-invisible-dry-shampoo-7716350.html</t>
         </is>
       </c>
-      <c r="E32" s="7" t="inlineStr"/>
-      <c r="F32" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr"/>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>7716350</t>
         </is>
       </c>
-      <c r="H32" s="7" t="inlineStr">
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -15655,40 +15655,40 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>Sublime Curl Activating Detangling Conditioner
 Condicionador Suave e Redefinidor de Caracóis
 150 ml</t>
         </is>
       </c>
-      <c r="D48" s="7" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/sublime-curl-activating-detangling-conditioner-5972162.html</t>
         </is>
       </c>
-      <c r="E48" s="7" t="inlineStr"/>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="E48" s="5" t="inlineStr"/>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
         <is>
           <t>5972162</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr">
+      <c r="H48" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -15815,40 +15815,40 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C52" s="7" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>Sublime Karité Moisturizing Smooting Shampoo
 Champô Hidratante Cabelo Seco e Muito Seco
 200 ml</t>
         </is>
       </c>
-      <c r="D52" s="7" t="inlineStr">
+      <c r="D52" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/sublime-karite-moisturizing-smooting-shampoo-8109682.html</t>
         </is>
       </c>
-      <c r="E52" s="7" t="inlineStr"/>
-      <c r="F52" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="E52" s="5" t="inlineStr"/>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
         <is>
           <t>8109682</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H52" s="5" t="inlineStr">
         <is>
           <t>34%</t>
         </is>
@@ -15935,40 +15935,40 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr">
         <is>
           <t>Sublime Karité Taming Nourishing Mask
 Máscara Nutritiva Cabelo Muito Seco
 200 ml</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/sublime-karite-taming-nourishing-mask-8109707.html</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr"/>
-      <c r="F55" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>8109707</t>
         </is>
       </c>
-      <c r="H55" s="7" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -17471,43 +17471,43 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Epitheliale Ultra Repair Cream SPF50+
 Creme Protetor Solar Reparador</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/epitheliale-ultra-repair-cream-spf50-412214.html</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>40 ml</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>8478836</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -17594,40 +17594,40 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Epitheliale Ultra Repair Serum VIT C+
 Sérum Luminosidade e Rugas Vitamina C
 30 ml</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/epitheliale-ultra-repair-serum-vit-c-8478841.html</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr"/>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>8478841</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -18728,40 +18728,40 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>Lip Stick
 Stick Lábios Hidratante e Reparador Pele Seca
 4 gr</t>
         </is>
       </c>
-      <c r="D49" s="7" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/lip-stick-5976847.html</t>
         </is>
       </c>
-      <c r="E49" s="7" t="inlineStr"/>
-      <c r="F49" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="E49" s="5" t="inlineStr"/>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
         <is>
           <t>5976847</t>
         </is>
       </c>
-      <c r="H49" s="7" t="inlineStr">
+      <c r="H49" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -18887,40 +18887,40 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C53" s="7" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>Protect Cream SPF50+
 Protetor Solar Creme Rosto Pele Seca
 40 ml</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D53" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-cream-spf50-5782489.html</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr"/>
-      <c r="F53" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr">
+      <c r="E53" s="5" t="inlineStr"/>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
         <is>
           <t>5782489</t>
         </is>
       </c>
-      <c r="H53" s="7" t="inlineStr">
+      <c r="H53" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -21243,17 +21243,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>Elgydium
 Escovilhão Interdentário Laranja
@@ -21261,23 +21261,23 @@
 1 un</t>
         </is>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/escovilhao-interdentario-laranja-8420655.html</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr"/>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="E50" s="3" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
         <is>
           <t>8420655</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H50" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -21487,40 +21487,40 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C56" s="7" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>Elgydium
 Fio Dentário Black
 1 un</t>
         </is>
       </c>
-      <c r="D56" s="7" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/fio-dentario-black-5786948.html</t>
         </is>
       </c>
-      <c r="E56" s="7" t="inlineStr"/>
-      <c r="F56" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr"/>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>5786948</t>
         </is>
       </c>
-      <c r="H56" s="7" t="inlineStr">
+      <c r="H56" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -22128,17 +22128,17 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C72" s="3" t="inlineStr">
+      <c r="C72" s="7" t="inlineStr">
         <is>
           <t>Eludril
 Intense Colutório Uso Diário
@@ -22146,23 +22146,23 @@
 500 ml</t>
         </is>
       </c>
-      <c r="D72" s="3" t="inlineStr">
+      <c r="D72" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/intense-colutorio-uso-diario-7181937.html</t>
         </is>
       </c>
-      <c r="E72" s="3" t="inlineStr"/>
-      <c r="F72" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G72" s="3" t="inlineStr">
+      <c r="E72" s="7" t="inlineStr"/>
+      <c r="F72" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
         <is>
           <t>7181937</t>
         </is>
       </c>
-      <c r="H72" s="3" t="inlineStr">
+      <c r="H72" s="7" t="inlineStr">
         <is>
           <t>Sem desconto</t>
         </is>
@@ -22693,17 +22693,17 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B86" s="7" t="inlineStr">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C86" s="7" t="inlineStr">
+      <c r="C86" s="3" t="inlineStr">
         <is>
           <t>Elgydium
 Refill Interdental Brushes ISO5
@@ -22711,23 +22711,23 @@
 3 un</t>
         </is>
       </c>
-      <c r="D86" s="7" t="inlineStr">
+      <c r="D86" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/refill-interdental-brushes-iso5-8547079.html</t>
         </is>
       </c>
-      <c r="E86" s="7" t="inlineStr"/>
-      <c r="F86" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G86" s="7" t="inlineStr">
+      <c r="E86" s="3" t="inlineStr"/>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
         <is>
           <t>8547079</t>
         </is>
       </c>
-      <c r="H86" s="7" t="inlineStr">
+      <c r="H86" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -22898,40 +22898,40 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B91" s="7" t="inlineStr">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C91" s="7" t="inlineStr">
+      <c r="C91" s="5" t="inlineStr">
         <is>
           <t>Elgydium
 Spray Cicallium
 15 ml</t>
         </is>
       </c>
-      <c r="D91" s="7" t="inlineStr">
+      <c r="D91" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/spray-cicallium-6637665.html</t>
         </is>
       </c>
-      <c r="E91" s="7" t="inlineStr"/>
-      <c r="F91" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G91" s="7" t="inlineStr">
+      <c r="E91" s="5" t="inlineStr"/>
+      <c r="F91" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
         <is>
           <t>6637665</t>
         </is>
       </c>
-      <c r="H91" s="7" t="inlineStr">
+      <c r="H91" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -23101,17 +23101,17 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="7" t="inlineStr">
-        <is>
-          <t>07/05/2026</t>
-        </is>
-      </c>
-      <c r="B96" s="7" t="inlineStr">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C96" s="7" t="inlineStr">
+      <c r="C96" s="3" t="inlineStr">
         <is>
           <t>Elgydium
 Trio Compact Interdental Brushes Fine Large
@@ -23119,23 +23119,23 @@
 1 un</t>
         </is>
       </c>
-      <c r="D96" s="7" t="inlineStr">
+      <c r="D96" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/trio-compact-interdental-brushes-fine-large-8414338.html</t>
         </is>
       </c>
-      <c r="E96" s="7" t="inlineStr"/>
-      <c r="F96" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G96" s="7" t="inlineStr">
+      <c r="E96" s="3" t="inlineStr"/>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
         <is>
           <t>8414338</t>
         </is>
       </c>
-      <c r="H96" s="7" t="inlineStr">
+      <c r="H96" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -23992,38 +23992,38 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Epitheliale Ultra Repair Cream SPF50+
 Creme Protetor Solar Reparador</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>40 ml</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>8478836</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/epitheliale-ultra-repair-cream-spf50-412214.html</t>
         </is>
@@ -26081,38 +26081,38 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="7" t="inlineStr">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B64" s="7" t="inlineStr">
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>Flax Volume Fine Hair Shampoo
 Champô Fibras de Linho BIO Volume Cabelo Fino</t>
         </is>
       </c>
-      <c r="C64" s="7" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="inlineStr">
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>5221797</t>
         </is>
       </c>
-      <c r="F64" s="7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/flax-volume-fine-hair-shampoo-343984.html</t>
         </is>

</xml_diff>